<commit_message>
data(templates): update labor review workbooks
</commit_message>
<xml_diff>
--- a/bieu_mau/Lao động giám đốc thẩm.xlsx
+++ b/bieu_mau/Lao động giám đốc thẩm.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LAPTOP-TUANDQ\Desktop\Quản lý tòa án - Project\biểu mẫu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QLTA-Project\bieu_mau\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA9F35BD-F7C9-4CA3-A797-1696F15F25A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC91671-E28A-4201-BD62-29C916C05CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{427023B4-7E91-432A-A15F-BC49B57D0662}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13290" xr2:uid="{427023B4-7E91-432A-A15F-BC49B57D0662}"/>
   </bookViews>
   <sheets>
     <sheet name="LaoDong_GDT" sheetId="1" r:id="rId1"/>
@@ -28,9 +28,6 @@
     <t>THỐNG KÊ THỤ LÝ VÀ GIẢI QUYẾT CÁC VỤ, VIỆC LAO ĐỘNG GIÁM ĐỐC THẨM</t>
   </si>
   <si>
-    <t>Mẫu 3C</t>
-  </si>
-  <si>
     <t>QUẢNG NGÃI</t>
   </si>
   <si>
@@ -134,6 +131,9 @@
   </si>
   <si>
     <t>Tổng cộng</t>
+  </si>
+  <si>
+    <t>Mẫu 5C</t>
   </si>
 </sst>
 </file>
@@ -144,21 +144,21 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="18"/>
       <color theme="3"/>
-      <name val="Calibri Light"/>
+      <name val="Times New Roman"/>
       <family val="2"/>
       <scheme val="major"/>
     </font>
@@ -166,7 +166,7 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -174,7 +174,7 @@
       <b/>
       <sz val="13"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -182,35 +182,35 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -218,7 +218,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -226,14 +226,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -241,14 +241,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -256,7 +256,7 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -264,14 +264,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -762,6 +762,36 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -770,36 +800,6 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1157,266 +1157,266 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA55BD0D-2600-4ED5-AAF4-8C796A8AF2C0}">
   <dimension ref="A1:AD8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" customWidth="1"/>
-    <col min="2" max="18" width="6.42578125" customWidth="1"/>
-    <col min="19" max="29" width="7.85546875" customWidth="1"/>
-    <col min="30" max="30" width="6.42578125" customWidth="1"/>
+    <col min="1" max="1" width="22.875" customWidth="1"/>
+    <col min="2" max="18" width="6.375" customWidth="1"/>
+    <col min="19" max="29" width="7.875" customWidth="1"/>
+    <col min="30" max="30" width="6.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" s="1" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
-      <c r="Y1" s="10" t="s">
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
+      <c r="P1" s="20"/>
+      <c r="Q1" s="20"/>
+      <c r="R1" s="20"/>
+      <c r="S1" s="20"/>
+      <c r="T1" s="20"/>
+      <c r="U1" s="20"/>
+      <c r="V1" s="20"/>
+      <c r="W1" s="20"/>
+      <c r="X1" s="20"/>
+      <c r="Y1" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z1" s="20"/>
+      <c r="AA1" s="20"/>
+      <c r="AB1" s="20"/>
+      <c r="AC1" s="20"/>
+      <c r="AD1" s="20"/>
+    </row>
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="Z1" s="10"/>
-      <c r="AA1" s="10"/>
-      <c r="AB1" s="10"/>
-      <c r="AC1" s="10"/>
-      <c r="AD1" s="10"/>
-    </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="B2" s="21"/>
+      <c r="C2" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
+      <c r="Y2" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
-      <c r="V2" s="12"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="Z2" s="12"/>
-      <c r="AA2" s="12"/>
-      <c r="AB2" s="12"/>
-      <c r="AC2" s="12"/>
-      <c r="AD2" s="12"/>
+      <c r="Z2" s="22"/>
+      <c r="AA2" s="22"/>
+      <c r="AB2" s="22"/>
+      <c r="AC2" s="22"/>
+      <c r="AD2" s="22"/>
     </row>
     <row r="3" spans="1:30" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="16" t="s">
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="16" t="s">
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="O3" s="17"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="18"/>
-      <c r="S3" s="16" t="s">
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
+      <c r="X3" s="19"/>
+      <c r="Y3" s="19"/>
+      <c r="Z3" s="19"/>
+      <c r="AA3" s="19"/>
+      <c r="AB3" s="19"/>
+      <c r="AC3" s="13"/>
+      <c r="AD3" s="14" t="s">
         <v>10</v>
-      </c>
-      <c r="T3" s="17"/>
-      <c r="U3" s="17"/>
-      <c r="V3" s="17"/>
-      <c r="W3" s="17"/>
-      <c r="X3" s="17"/>
-      <c r="Y3" s="17"/>
-      <c r="Z3" s="17"/>
-      <c r="AA3" s="17"/>
-      <c r="AB3" s="17"/>
-      <c r="AC3" s="18"/>
-      <c r="AD3" s="13" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:30" s="1" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14"/>
-      <c r="B4" s="16" t="s">
+      <c r="A4" s="18"/>
+      <c r="B4" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="13"/>
+      <c r="D4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="16" t="s">
+      <c r="E4" s="13"/>
+      <c r="F4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="18"/>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="19"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="17"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="16" t="s">
+      <c r="J4" s="13"/>
+      <c r="K4" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="18"/>
-      <c r="K4" s="16" t="s">
+      <c r="L4" s="13"/>
+      <c r="M4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="N4" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="L4" s="18"/>
-      <c r="M4" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="N4" s="19" t="s">
+      <c r="O4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="O4" s="19" t="s">
+      <c r="P4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="P4" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q4" s="21" t="s">
+      <c r="R4" s="17"/>
+      <c r="S4" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="R4" s="22"/>
-      <c r="S4" s="16" t="s">
+      <c r="T4" s="13"/>
+      <c r="U4" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="T4" s="18"/>
-      <c r="U4" s="13" t="s">
+      <c r="V4" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="V4" s="13" t="s">
+      <c r="W4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="W4" s="19" t="s">
+      <c r="X4" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="X4" s="19" t="s">
+      <c r="Y4" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="Y4" s="19" t="s">
+      <c r="Z4" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="Z4" s="19" t="s">
+      <c r="AA4" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="AA4" s="19" t="s">
+      <c r="AB4" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="AB4" s="19" t="s">
+      <c r="AC4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="AC4" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="AD4" s="14"/>
+      <c r="AD4" s="18"/>
     </row>
     <row r="5" spans="1:30" s="1" customFormat="1" ht="145.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="15"/>
       <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="D5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="F5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="H5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="K5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="K5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
-      <c r="P5" s="20"/>
-      <c r="Q5" s="3" t="s">
+      <c r="R5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="R5" s="3" t="s">
+      <c r="S5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="S5" s="3" t="s">
+      <c r="T5" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="T5" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="U5" s="15"/>
       <c r="V5" s="15"/>
-      <c r="W5" s="20"/>
-      <c r="X5" s="20"/>
-      <c r="Y5" s="20"/>
-      <c r="Z5" s="20"/>
-      <c r="AA5" s="20"/>
-      <c r="AB5" s="20"/>
-      <c r="AC5" s="20"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
+      <c r="Y5" s="11"/>
+      <c r="Z5" s="11"/>
+      <c r="AA5" s="11"/>
+      <c r="AB5" s="11"/>
+      <c r="AC5" s="11"/>
       <c r="AD5" s="15"/>
     </row>
     <row r="6" spans="1:30" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
@@ -1513,7 +1513,7 @@
     </row>
     <row r="7" spans="1:30" s="1" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1579,6 +1579,28 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:X1"/>
+    <mergeCell ref="Y1:AD1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:X2"/>
+    <mergeCell ref="Y2:AD2"/>
+    <mergeCell ref="S3:AC3"/>
+    <mergeCell ref="AD3:AD5"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="I3:M3"/>
+    <mergeCell ref="N3:R3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="O4:O5"/>
+    <mergeCell ref="P4:P5"/>
     <mergeCell ref="Z4:Z5"/>
     <mergeCell ref="AA4:AA5"/>
     <mergeCell ref="AB4:AB5"/>
@@ -1589,28 +1611,6 @@
     <mergeCell ref="W4:W5"/>
     <mergeCell ref="X4:X5"/>
     <mergeCell ref="Y4:Y5"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="O4:O5"/>
-    <mergeCell ref="P4:P5"/>
-    <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="I3:M3"/>
-    <mergeCell ref="N3:R3"/>
-    <mergeCell ref="S3:AC3"/>
-    <mergeCell ref="AD3:AD5"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:X1"/>
-    <mergeCell ref="Y1:AD1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:X2"/>
-    <mergeCell ref="Y2:AD2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>